<commit_message>
docs: sincroniza documentacao e corrige anotacao da cacamba no dicionario
- GUIA: Problema #1 (esgoto V00312-V00316) e #6 (docs) marcados resolvidos;
  rotulo de V00900 corrigido para "alfabetizados 15+"; tests/ deixa de ser
  descrita como vazia (16 testes); De-Para sem o aviso do esgoto.
- Relatorio_Integridade: esgoto e "variaveis vs dicionario" resolvidos;
  contagem de testes ajustada (16 passam).
- Dicionario_IBGE_Oficial: V00398 (cacamba) reanotada como INADEQUADA
  (numerador) por fidelidade ao IVS-BH 2012, removendo o residuo do bug ja
  revertido ("excluir - bug atual"); LEIA-ME esclarece que as colunas de
  adequacao sao anotacao do projeto, nao verbatim do IBGE.
</commit_message>
<xml_diff>
--- a/docs/Apresentacoes_IVS/Dicionario_IBGE_Oficial_Variaveis_do_Projeto.xlsx
+++ b/docs/Apresentacoes_IVS/Dicionario_IBGE_Oficial_Variaveis_do_Projeto.xlsx
@@ -478,7 +478,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Recorte do dicionário oficial do IBGE (dicionario_de_dados_agregados_por_setores_censitarios_20260520.xlsx, baixado de ftp.ibge.gov.br em 18/06/2026) contendo APENAS as variáveis usadas no projeto IVS/Censo 2022. As descrições da coluna "Descricao_oficial_IBGE" são verbatim do IBGE. A coluna "Adequacao_saneamento" marca, para água/esgoto/lixo, quais categorias são adequadas (excluídas do numerador) e quais são inadequadas (entram no numerador). ATENÇÃO: V00398 (caçamba de serviço de limpeza) é COLETA ADEQUADA e NÃO deve compor pct_lixo_inad — numerador correto = V00399+V00400+V00401+V00402.</t>
+          <t>Recorte do dicionario oficial do IBGE (dicionario_de_dados_agregados_por_setores_censitarios_20260520.xlsx, baixado de ftp.ibge.gov.br em 18/06/2026) contendo APENAS as variaveis usadas no projeto IVS/Censo 2022. As descricoes da coluna "Descricao_oficial_IBGE" sao verbatim do IBGE; as colunas "Papel_no_projeto_IVS" e "Adequacao_saneamento" sao ANOTACOES DO PROJETO (nao do IBGE). A coluna "Adequacao_saneamento" marca, para agua/esgoto/lixo, quais categorias entram (inadequada) ou nao (adequada) no numerador, conforme a metodologia do IVS-BH 2012 que o projeto reproduz. NOTA V00398 (cacamba de servico de limpeza): por FIDELIDADE ao IVS-BH 2012 (docs/Calculo IVS2012.docx, Tabela 3 = V037 no Censo 2010) a caçamba e contada como lixo INADEQUADO e ENTRA no numerador de pct_lixo_inad (V00398+V00399+V00400+V00401+V00402); so a coleta porta-a-porta V00397 e adequada. A leitura moderna (IBGE/OMS: caçamba = coleta adequada) e uma divergencia legitima, mas seria um upgrade metodologico a decidir com a orientadora — nao o padrao atual. Decisao consolidada em 18/06/2026.</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1411,12 +1411,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>Lixo — coleta ADEQUADA (caçamba de serviço de limpeza). *** NÃO é inadequado — não deve entrar no numerador ***</t>
+          <t>Lixo — contado como INADEQUADO por fidelidade ao IVS-BH 2012 (so a coleta porta-a-porta V00397 e adequada). ENTRA no numerador de pct_lixo_inad. Divergencia moderna (IBGE/OMS: adequada) seria upgrade a decidir com a orientadora.</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>ADEQUADA (excluir — bug atual)</t>
+          <t>INADEQUADA (numerador) — por fidelidade ao IVS-BH 2012; ver NOTA no LEIA-ME</t>
         </is>
       </c>
     </row>

</xml_diff>